<commit_message>
data: EEX prices 2026-05-13
</commit_message>
<xml_diff>
--- a/data/eex_prix.xlsx
+++ b/data/eex_prix.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,1386 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>53.79</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>50.77</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>53.67</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>58.28</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>92.41</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>23</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>68.17</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>78.39</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>24.04</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>32.01</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>68.65000000000001</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>74.38</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ELEC-May-2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>40.03</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ELEC-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>25.06</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ELEC-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>40.78</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ELEC-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>37.63</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ELEC-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>52.62</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ELEC-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>71.02</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ELEC-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>97.62</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ELEC-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>94.45</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ELEC-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>106.85</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ELEC-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Power FR Baseload</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Power FR Peakload</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>60.23</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Power FR Peakload</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>59</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Power FR Peakload</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>62.63</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Power FR Peakload</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>67.75</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>37.295</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>28.011</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>23.816</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>44.502</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>35.794</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>34.397</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>34.631</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>33.35</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>26.618</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>25.553</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>26.568</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>26.401</v>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2029</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>22.964</v>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2029</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>22.749</v>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2029</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2030</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>24.192</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2030</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>22.503</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2027</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Natural Gas TTF</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>34.809</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: EEX prices 2026-05-14
</commit_message>
<xml_diff>
--- a/data/eex_prix.xlsx
+++ b/data/eex_prix.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Natural Gas PEG" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Natural Gas TTF'!$A$1:$E$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1196,8 +1196,683 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>54.01</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>50.99</v>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>53.99</v>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>92.53</v>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>23.46</v>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>32.66</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>67.91</v>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>78.73999999999999</v>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>24.14</v>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>32.15</v>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>68.95</v>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>74.81999999999999</v>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-May-2026</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>38.68</v>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>25.34</v>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>41.28</v>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>37.93</v>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>70.84</v>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>97.42</v>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>94.81999999999999</v>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>106.99</v>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>102.48</v>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>60.58</v>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>59.63</v>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>62.61</v>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>68.27</v>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E28"/>
+  <autoFilter ref="A1:E55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1257,7 +1932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1744,8 +2419,958 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>36.445</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>27.399</v>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>23.475</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n">
+        <v>22.131</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="n">
+        <v>43.455</v>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="n">
+        <v>35.202</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>33.684</v>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="n">
+        <v>33.579</v>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>32.516</v>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="n">
+        <v>26.598</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>24.697</v>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>25.831</v>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>26.444</v>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2029</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="n">
+        <v>22.442</v>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2029</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D34" s="7" t="n">
+        <v>22.227</v>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2029</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="n">
+        <v>22.842</v>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2030</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>24.06</v>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2030</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="n">
+        <v>22.265</v>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2030</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>20.125</v>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2030</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="n">
+        <v>22.117</v>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2026</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="n">
+        <v>45.944</v>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="n">
+        <v>46.16</v>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="n">
+        <v>46.307</v>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D43" s="8" t="n">
+        <v>46.233</v>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="n">
+        <v>46.242</v>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D45" s="8" t="n">
+        <v>45.317</v>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="n">
+        <v>44.571</v>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D47" s="8" t="n">
+        <v>44.564</v>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>44.019</v>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="n">
+        <v>44.164</v>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Mar-2027</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>42.25</v>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Apr-2027</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="n">
+        <v>36.543</v>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2027</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="n">
+        <v>34.759</v>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2027</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>34.319</v>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2027</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="n">
+        <v>33.549</v>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2027</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="n">
+        <v>33.655</v>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2027</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>33.854</v>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2027</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="n">
+        <v>33.206</v>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E19"/>
+  <autoFilter ref="A1:E57"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: EEX prices 2026-05-15
</commit_message>
<xml_diff>
--- a/data/eex_prix.xlsx
+++ b/data/eex_prix.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Natural Gas PEG" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$82</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Natural Gas TTF'!$A$1:$E$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1871,8 +1871,683 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="n">
+        <v>54.59</v>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="n">
+        <v>50.92</v>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="n">
+        <v>53.93</v>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="n">
+        <v>58.74</v>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>92.77</v>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="n">
+        <v>24.63</v>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>33.43</v>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="n">
+        <v>68.05</v>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>78.98999999999999</v>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="n">
+        <v>23.98</v>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>31.98</v>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="n">
+        <v>68.73</v>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>74.73999999999999</v>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-May-2026</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="n">
+        <v>37.69</v>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>23.83</v>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>37.69</v>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="n">
+        <v>54.54</v>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>71.52</v>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="n">
+        <v>98.31999999999999</v>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>95.25</v>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>107.22</v>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="n">
+        <v>61.1</v>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>59.7</v>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>68.45</v>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E55"/>
+  <autoFilter ref="A1:E82"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1932,7 +2607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3369,8 +4044,958 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="n">
+        <v>35.866</v>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="n">
+        <v>26.858</v>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>23.053</v>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="n">
+        <v>22.125</v>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>43.158</v>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="n">
+        <v>34.54</v>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>32.967</v>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="n">
+        <v>32.944</v>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>31.966</v>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="n">
+        <v>26.063</v>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>24.184</v>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="n">
+        <v>25.268</v>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>25.686</v>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2029</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="n">
+        <v>22.055</v>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2029</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="n">
+        <v>21.842</v>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2029</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="n">
+        <v>22.662</v>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2030</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>23.918</v>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2030</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="n">
+        <v>22.335</v>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2030</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>20.173</v>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2030</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="n">
+        <v>22.116</v>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2026</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="n">
+        <v>45.944</v>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D79" s="8" t="n">
+        <v>46.894</v>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="n">
+        <v>46.971</v>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D81" s="8" t="n">
+        <v>46.819</v>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="n">
+        <v>46.749</v>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="n">
+        <v>45.398</v>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>44.652</v>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="n">
+        <v>44.645</v>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="n">
+        <v>43.716</v>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="n">
+        <v>43.864</v>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Mar-2027</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="n">
+        <v>41.961</v>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Apr-2027</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="n">
+        <v>35.858</v>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2027</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="n">
+        <v>34.104</v>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2027</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="n">
+        <v>33.672</v>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2027</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="n">
+        <v>32.834</v>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2027</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="n">
+        <v>32.938</v>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2027</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="n">
+        <v>33.133</v>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2027</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="n">
+        <v>32.568</v>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E57"/>
+  <autoFilter ref="A1:E95"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: EEX prices 2026-05-18
</commit_message>
<xml_diff>
--- a/data/eex_prix.xlsx
+++ b/data/eex_prix.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Natural Gas PEG" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Natural Gas TTF'!$A$1:$E$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2546,8 +2546,683 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D83" s="8" t="n">
+        <v>55.75</v>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D84" s="7" t="n">
+        <v>51.65</v>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D85" s="8" t="n">
+        <v>54.36</v>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="n">
+        <v>59.17</v>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D87" s="8" t="n">
+        <v>94.77</v>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="n">
+        <v>25.47</v>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D89" s="8" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="n">
+        <v>69.26000000000001</v>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D91" s="8" t="n">
+        <v>79.40000000000001</v>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="n">
+        <v>24.56</v>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D93" s="8" t="n">
+        <v>32.68</v>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="n">
+        <v>69.95999999999999</v>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D95" s="8" t="n">
+        <v>75.34</v>
+      </c>
+      <c r="E95" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-May-2026</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="n">
+        <v>40.29</v>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="n">
+        <v>24.14</v>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="n">
+        <v>40.46</v>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="n">
+        <v>38.42</v>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>58.58</v>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="n">
+        <v>73.59</v>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="n">
+        <v>100.54</v>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="n">
+        <v>96.89</v>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="n">
+        <v>109.6</v>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D105" s="8" t="n">
+        <v>104.98</v>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="n">
+        <v>61.85</v>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D107" s="8" t="n">
+        <v>60.09</v>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="n">
+        <v>63</v>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D109" s="8" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E82"/>
+  <autoFilter ref="A1:E109"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2607,7 +3282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E95"/>
+  <dimension ref="A1:E133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4994,8 +5669,958 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="n">
+        <v>37.08</v>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D97" s="8" t="n">
+        <v>27.239</v>
+      </c>
+      <c r="E97" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="n">
+        <v>23.315</v>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D99" s="8" t="n">
+        <v>22.025</v>
+      </c>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="n">
+        <v>45.307</v>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D101" s="8" t="n">
+        <v>35.596</v>
+      </c>
+      <c r="E101" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="n">
+        <v>33.848</v>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D103" s="8" t="n">
+        <v>33.731</v>
+      </c>
+      <c r="E103" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="n">
+        <v>32.661</v>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D105" s="8" t="n">
+        <v>26.361</v>
+      </c>
+      <c r="E105" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D106" s="7" t="n">
+        <v>24.468</v>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D107" s="8" t="n">
+        <v>25.528</v>
+      </c>
+      <c r="E107" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D108" s="7" t="n">
+        <v>26.137</v>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2029</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D109" s="8" t="n">
+        <v>22.314</v>
+      </c>
+      <c r="E109" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2029</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="n">
+        <v>22.099</v>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2029</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="n">
+        <v>22.759</v>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2030</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D112" s="7" t="n">
+        <v>23.904</v>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2030</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D113" s="8" t="n">
+        <v>22.176</v>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2030</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="n">
+        <v>20.022</v>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2030</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="n">
+        <v>22.041</v>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2026</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="n">
+        <v>45.944</v>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="n">
+        <v>49.428</v>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="n">
+        <v>49.546</v>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D119" s="8" t="n">
+        <v>49.441</v>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="n">
+        <v>48.997</v>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="n">
+        <v>47.777</v>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="n">
+        <v>47.007</v>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D123" s="8" t="n">
+        <v>47.003</v>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D124" s="7" t="n">
+        <v>45.913</v>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D125" s="8" t="n">
+        <v>46.04</v>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Mar-2027</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D126" s="7" t="n">
+        <v>44.038</v>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Apr-2027</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D127" s="8" t="n">
+        <v>36.957</v>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2027</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D128" s="7" t="n">
+        <v>35.146</v>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2027</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="n">
+        <v>34.699</v>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2027</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="n">
+        <v>33.712</v>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2027</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D131" s="8" t="n">
+        <v>33.819</v>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2027</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D132" s="7" t="n">
+        <v>34.02</v>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2027</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D133" s="8" t="n">
+        <v>33.36</v>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E95"/>
+  <autoFilter ref="A1:E133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: EEX prices 2026-05-19
</commit_message>
<xml_diff>
--- a/data/eex_prix.xlsx
+++ b/data/eex_prix.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Natural Gas PEG" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$136</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Natural Gas TTF'!$A$1:$E$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$171</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3221,8 +3221,683 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D110" s="7" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D111" s="8" t="n">
+        <v>51.39</v>
+      </c>
+      <c r="E111" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D112" s="7" t="n">
+        <v>54.45</v>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D113" s="8" t="n">
+        <v>58.92</v>
+      </c>
+      <c r="E113" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D114" s="7" t="n">
+        <v>95.11</v>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D115" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="E115" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="n">
+        <v>33.48</v>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D117" s="8" t="n">
+        <v>68.55</v>
+      </c>
+      <c r="E117" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="n">
+        <v>78.14</v>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D119" s="8" t="n">
+        <v>24.72</v>
+      </c>
+      <c r="E119" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D120" s="7" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D121" s="8" t="n">
+        <v>69.89</v>
+      </c>
+      <c r="E121" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D122" s="7" t="n">
+        <v>75.45999999999999</v>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-May-2026</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D123" s="8" t="n">
+        <v>40.79</v>
+      </c>
+      <c r="E123" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D124" s="7" t="n">
+        <v>25.05</v>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D125" s="8" t="n">
+        <v>41.04</v>
+      </c>
+      <c r="E125" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D126" s="7" t="n">
+        <v>38.47</v>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D127" s="8" t="n">
+        <v>59.64</v>
+      </c>
+      <c r="E127" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D128" s="7" t="n">
+        <v>74.90000000000001</v>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D129" s="8" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="E129" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D130" s="7" t="n">
+        <v>97.70999999999999</v>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D131" s="8" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="E131" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D132" s="7" t="n">
+        <v>105.84</v>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D133" s="8" t="n">
+        <v>62.22</v>
+      </c>
+      <c r="E133" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D134" s="7" t="n">
+        <v>59.73</v>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D135" s="8" t="n">
+        <v>62.9</v>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D136" s="7" t="n">
+        <v>68.52</v>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E109"/>
+  <autoFilter ref="A1:E136"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3282,7 +3957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E133"/>
+  <dimension ref="A1:E171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6619,8 +7294,958 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D134" s="7" t="n">
+        <v>37.23</v>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D135" s="8" t="n">
+        <v>27.315</v>
+      </c>
+      <c r="E135" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D136" s="7" t="n">
+        <v>23.381</v>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="n">
+        <v>22.025</v>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D138" s="7" t="n">
+        <v>45.502</v>
+      </c>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D139" s="8" t="n">
+        <v>35.668</v>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D140" s="7" t="n">
+        <v>34.061</v>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D141" s="8" t="n">
+        <v>33.853</v>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D142" s="7" t="n">
+        <v>32.791</v>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D143" s="8" t="n">
+        <v>26.457</v>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D144" s="7" t="n">
+        <v>24.558</v>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D145" s="8" t="n">
+        <v>25.503</v>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D146" s="7" t="n">
+        <v>26.24</v>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2029</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D147" s="8" t="n">
+        <v>22.365</v>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2029</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D148" s="7" t="n">
+        <v>22.148</v>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2029</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D149" s="8" t="n">
+        <v>22.811</v>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2030</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D150" s="7" t="n">
+        <v>23.945</v>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2030</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D151" s="8" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2030</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D152" s="7" t="n">
+        <v>20.024</v>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2030</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="n">
+        <v>21.973</v>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2026</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D154" s="7" t="n">
+        <v>45.944</v>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="n">
+        <v>49.521</v>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D156" s="7" t="n">
+        <v>49.713</v>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="n">
+        <v>49.569</v>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D158" s="7" t="n">
+        <v>49.442</v>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D159" s="8" t="n">
+        <v>47.949</v>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D160" s="7" t="n">
+        <v>47.381</v>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D161" s="8" t="n">
+        <v>47.378</v>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D162" s="7" t="n">
+        <v>46.115</v>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D163" s="8" t="n">
+        <v>46.239</v>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Mar-2027</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D164" s="7" t="n">
+        <v>44.223</v>
+      </c>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Apr-2027</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D165" s="8" t="n">
+        <v>37.035</v>
+      </c>
+      <c r="E165" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2027</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D166" s="7" t="n">
+        <v>35.216</v>
+      </c>
+      <c r="E166" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2027</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D167" s="8" t="n">
+        <v>34.767</v>
+      </c>
+      <c r="E167" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2027</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D168" s="7" t="n">
+        <v>33.924</v>
+      </c>
+      <c r="E168" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2027</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D169" s="8" t="n">
+        <v>34.032</v>
+      </c>
+      <c r="E169" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2027</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D170" s="7" t="n">
+        <v>34.234</v>
+      </c>
+      <c r="E170" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2027</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D171" s="8" t="n">
+        <v>33.483</v>
+      </c>
+      <c r="E171" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E133"/>
+  <autoFilter ref="A1:E171"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
data: EEX prices 2026-05-20
</commit_message>
<xml_diff>
--- a/data/eex_prix.xlsx
+++ b/data/eex_prix.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Natural Gas PEG" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Power FR'!$A$1:$E$163</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Natural Gas TTF'!$A$1:$E$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Natural Gas PEG'!$A$1:$E$209</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E136"/>
+  <dimension ref="A1:E163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3896,8 +3896,683 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D137" s="8" t="n">
+        <v>55.74</v>
+      </c>
+      <c r="E137" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D138" s="7" t="n">
+        <v>51.66</v>
+      </c>
+      <c r="E138" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D139" s="8" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="E139" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D140" s="7" t="n">
+        <v>58.7</v>
+      </c>
+      <c r="E140" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D141" s="8" t="n">
+        <v>96.04000000000001</v>
+      </c>
+      <c r="E141" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D142" s="7" t="n">
+        <v>25.4</v>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D143" s="8" t="n">
+        <v>33.75</v>
+      </c>
+      <c r="E143" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D144" s="7" t="n">
+        <v>68.33</v>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D145" s="8" t="n">
+        <v>78.66</v>
+      </c>
+      <c r="E145" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D146" s="7" t="n">
+        <v>24.82</v>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D147" s="8" t="n">
+        <v>32.94</v>
+      </c>
+      <c r="E147" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D148" s="7" t="n">
+        <v>70.23</v>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D149" s="8" t="n">
+        <v>75.25</v>
+      </c>
+      <c r="E149" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-May-2026</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D150" s="7" t="n">
+        <v>41.97</v>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D151" s="8" t="n">
+        <v>27.15</v>
+      </c>
+      <c r="E151" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D152" s="7" t="n">
+        <v>46.05</v>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D153" s="8" t="n">
+        <v>40.72</v>
+      </c>
+      <c r="E153" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D154" s="7" t="n">
+        <v>59.71</v>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D155" s="8" t="n">
+        <v>73.95</v>
+      </c>
+      <c r="E155" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D156" s="7" t="n">
+        <v>104.34</v>
+      </c>
+      <c r="E156" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D157" s="8" t="n">
+        <v>99.94</v>
+      </c>
+      <c r="E157" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>ELEC-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D158" s="7" t="n">
+        <v>112.01</v>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>ELEC-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D159" s="8" t="n">
+        <v>107.29</v>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D160" s="7" t="n">
+        <v>62.36</v>
+      </c>
+      <c r="E160" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D161" s="8" t="n">
+        <v>60.25</v>
+      </c>
+      <c r="E161" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D162" s="7" t="n">
+        <v>62.93</v>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>PEAK-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D163" s="8" t="n">
+        <v>68.40000000000001</v>
+      </c>
+      <c r="E163" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E136"/>
+  <autoFilter ref="A1:E163"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3957,7 +4632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E171"/>
+  <dimension ref="A1:E209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8244,8 +8919,958 @@
         </is>
       </c>
     </row>
+    <row r="172">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2027</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D172" s="7" t="n">
+        <v>37.495</v>
+      </c>
+      <c r="E172" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2028</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D173" s="8" t="n">
+        <v>27.189</v>
+      </c>
+      <c r="E173" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2029</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D174" s="7" t="n">
+        <v>23.638</v>
+      </c>
+      <c r="E174" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-CAL-2030</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>CAL</t>
+        </is>
+      </c>
+      <c r="D175" s="8" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="E175" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2027</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D176" s="7" t="n">
+        <v>46.46</v>
+      </c>
+      <c r="E176" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2027</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D177" s="8" t="n">
+        <v>35.692</v>
+      </c>
+      <c r="E177" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2027</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D178" s="7" t="n">
+        <v>34.083</v>
+      </c>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2027</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D179" s="8" t="n">
+        <v>33.92</v>
+      </c>
+      <c r="E179" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2028</t>
+        </is>
+      </c>
+      <c r="C180" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D180" s="7" t="n">
+        <v>32.794</v>
+      </c>
+      <c r="E180" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2028</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D181" s="8" t="n">
+        <v>26.252</v>
+      </c>
+      <c r="E181" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2028</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D182" s="7" t="n">
+        <v>24.406</v>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B183" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2028</t>
+        </is>
+      </c>
+      <c r="C183" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D183" s="8" t="n">
+        <v>25.353</v>
+      </c>
+      <c r="E183" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2029</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D184" s="7" t="n">
+        <v>26.481</v>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B185" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2029</t>
+        </is>
+      </c>
+      <c r="C185" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D185" s="8" t="n">
+        <v>22.623</v>
+      </c>
+      <c r="E185" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2029</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D186" s="7" t="n">
+        <v>22.404</v>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B187" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2029</t>
+        </is>
+      </c>
+      <c r="C187" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D187" s="8" t="n">
+        <v>23.096</v>
+      </c>
+      <c r="E187" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q1-2030</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D188" s="7" t="n">
+        <v>24.029</v>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B189" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q2-2030</t>
+        </is>
+      </c>
+      <c r="C189" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D189" s="8" t="n">
+        <v>22.317</v>
+      </c>
+      <c r="E189" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Q3-2030</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D190" s="7" t="n">
+        <v>20.115</v>
+      </c>
+      <c r="E190" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B191" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Q4-2030</t>
+        </is>
+      </c>
+      <c r="C191" s="5" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="D191" s="8" t="n">
+        <v>21.982</v>
+      </c>
+      <c r="E191" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2026</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D192" s="7" t="n">
+        <v>45.944</v>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B193" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2026</t>
+        </is>
+      </c>
+      <c r="C193" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D193" s="8" t="n">
+        <v>51.148</v>
+      </c>
+      <c r="E193" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2026</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D194" s="7" t="n">
+        <v>51.259</v>
+      </c>
+      <c r="E194" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B195" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2026</t>
+        </is>
+      </c>
+      <c r="C195" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D195" s="8" t="n">
+        <v>51.172</v>
+      </c>
+      <c r="E195" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2026</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D196" s="7" t="n">
+        <v>50.87</v>
+      </c>
+      <c r="E196" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B197" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2026</t>
+        </is>
+      </c>
+      <c r="C197" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D197" s="8" t="n">
+        <v>49.274</v>
+      </c>
+      <c r="E197" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Nov-2026</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D198" s="7" t="n">
+        <v>48.698</v>
+      </c>
+      <c r="E198" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B199" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Dec-2026</t>
+        </is>
+      </c>
+      <c r="C199" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D199" s="8" t="n">
+        <v>48.696</v>
+      </c>
+      <c r="E199" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jan-2027</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D200" s="7" t="n">
+        <v>47.095</v>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B201" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Feb-2027</t>
+        </is>
+      </c>
+      <c r="C201" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D201" s="8" t="n">
+        <v>47.209</v>
+      </c>
+      <c r="E201" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Mar-2027</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D202" s="7" t="n">
+        <v>45.149</v>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B203" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Apr-2027</t>
+        </is>
+      </c>
+      <c r="C203" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D203" s="8" t="n">
+        <v>37.06</v>
+      </c>
+      <c r="E203" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-May-2027</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D204" s="7" t="n">
+        <v>35.24</v>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B205" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Jun-2027</t>
+        </is>
+      </c>
+      <c r="C205" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D205" s="8" t="n">
+        <v>34.79</v>
+      </c>
+      <c r="E205" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Jul-2027</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D206" s="7" t="n">
+        <v>33.946</v>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B207" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Aug-2027</t>
+        </is>
+      </c>
+      <c r="C207" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D207" s="8" t="n">
+        <v>34.054</v>
+      </c>
+      <c r="E207" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>GAZ-Sep-2027</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D208" s="7" t="n">
+        <v>34.256</v>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="B209" s="5" t="inlineStr">
+        <is>
+          <t>GAZ-Oct-2027</t>
+        </is>
+      </c>
+      <c r="C209" s="5" t="inlineStr">
+        <is>
+          <t>MTH</t>
+        </is>
+      </c>
+      <c r="D209" s="8" t="n">
+        <v>33.55</v>
+      </c>
+      <c r="E209" s="5" t="inlineStr">
+        <is>
+          <t>Settlement</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E171"/>
+  <autoFilter ref="A1:E209"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>